<commit_message>
final next peak results
</commit_message>
<xml_diff>
--- a/PowerTest/PowerTest.xlsx
+++ b/PowerTest/PowerTest.xlsx
@@ -3916,7 +3916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4525,7 +4525,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>6034009</v>
+        <v>1106662</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -4539,34 +4539,38 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Nguyen MS</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>Geoffrey Gilbert9217</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BIKES &amp;#11088;&amp;#65039;</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>12:26.274</t>
+          <t>12:22.824</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>328</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>47.195</t>
+          <t>43.745</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>5393539</v>
+        <v>6034009</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -4580,34 +4584,34 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Carsten Jensen</t>
+          <t>Nguyen MS</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>13:48.454</t>
+          <t>12:26.274</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>313</t>
+          <t>223</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>02:09.375</t>
+          <t>47.195</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>6829675</v>
+        <v>1017356</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -4621,34 +4625,38 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Anders Stagsted</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>Nick Overkamp</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>WTOS</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>14:06.444</t>
+          <t>13:35.592</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>283</t>
+          <t>297</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>02:27.365</t>
+          <t>01:56.513</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1170121</v>
+        <v>5393539</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -4662,34 +4670,34 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Reona MTR</t>
+          <t>Carsten Jensen</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>14:41.692</t>
+          <t>13:48.454</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>265</t>
+          <t>313</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>03:02.613</t>
+          <t>02:09.375</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>718605</v>
+        <v>6829675</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -4703,151 +4711,454 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>I Cant ride</t>
+          <t>Anders Stagsted</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>14:43.183</t>
+          <t>14:06.444</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>283</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>03:04.104</t>
+          <t>02:27.365</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>779638</v>
+        <v>990876</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Tiana Abel</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t xml:space="preserve">Pete Connor (TNP) </t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Team Not Pogi</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>14:49.694</t>
+          <t>14:28.486</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>322</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>00.000</t>
+          <t>02:49.407</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>4651254</v>
+        <v>1170121</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Arjen De Jonge</t>
+          <t>Reona MTR</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>16:04.310</t>
+          <t>14:41.692</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>265</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>01:14.616</t>
+          <t>03:02.613</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1427961</v>
+        <v>718605</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Rob Koops</t>
+          <t>I Cant ride</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
+          <t>14:43.183</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>03:04.104</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>4177429</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F F </t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L&amp;rsquo;Equipe Provence</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>13:47.095</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>192</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>00.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>3084196</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darin Mills </t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>DIRT</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>13:58.271</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>288</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>11.176</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>779638</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Tiana Abel</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>14:49.694</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>192</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>01:02.599</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>4651254</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Arjen De Jonge</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>16:04.310</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>02:17.215</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>560748</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Travis Lewis</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>DIRT</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>16:10.475</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>218</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>02:23.380</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>458457</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Bart Van De Ven8888</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>17:45.141</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>288</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>03:58.046</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1427961</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Rob Koops</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>18:15.800</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>229</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>03:26.106</t>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>04:28.705</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update to headers on power test
</commit_message>
<xml_diff>
--- a/PowerTest/PowerTest.xlsx
+++ b/PowerTest/PowerTest.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>W/Kg</t>
+          <t>W/kg</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>W/Kg</t>
+          <t>W/kg</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>W/Kg</t>
+          <t>W/kg</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -3957,7 +3957,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>W/Kg</t>
+          <t>W/kg</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">

</xml_diff>